<commit_message>
docs: update example input
</commit_message>
<xml_diff>
--- a/docs/PARSE_TABLE_LL1.xlsx
+++ b/docs/PARSE_TABLE_LL1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nk/Documents/repos/PascalCompiler/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB1496F2-2782-D444-A13F-F35D2DBC212F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{332D9AF5-D737-064A-848A-F22BA869E027}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="200" yWindow="1080" windowWidth="33800" windowHeight="20940" xr2:uid="{A78E9B41-F319-8640-B78C-83646029D234}"/>
+    <workbookView xWindow="200" yWindow="1080" windowWidth="33800" windowHeight="20940" activeTab="1" xr2:uid="{A78E9B41-F319-8640-B78C-83646029D234}"/>
   </bookViews>
   <sheets>
     <sheet name="LL(1) Grammar" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="178">
   <si>
     <t>Productions</t>
   </si>
@@ -568,6 +568,9 @@
   </si>
   <si>
     <t>Term'</t>
+  </si>
+  <si>
+    <t>.</t>
   </si>
 </sst>
 </file>
@@ -634,9 +637,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -666,10 +666,13 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1007,679 +1010,679 @@
   <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.6640625" style="10" customWidth="1"/>
-    <col min="2" max="2" width="82.6640625" style="10" customWidth="1"/>
-    <col min="3" max="3" width="95.6640625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="49" style="8" customWidth="1"/>
+    <col min="1" max="1" width="6.6640625" style="9" customWidth="1"/>
+    <col min="2" max="2" width="82.6640625" style="9" customWidth="1"/>
+    <col min="3" max="3" width="95.6640625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="49" style="7" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="3" t="s">
+      <c r="B1" s="14"/>
+      <c r="C1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A2" s="8">
+      <c r="A2" s="7">
         <v>1</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="6" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" s="8">
+      <c r="A3" s="7">
         <v>2</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A4" s="8">
+      <c r="A4" s="7">
         <v>3</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="6" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5" s="8">
+      <c r="A5" s="7">
         <v>4</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="6" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A6" s="8">
+      <c r="A6" s="7">
         <v>5</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="6" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A7" s="8">
+      <c r="A7" s="7">
         <v>6</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="6" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A8" s="8">
+      <c r="A8" s="7">
         <v>7</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="6" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="51" x14ac:dyDescent="0.2">
-      <c r="A9" s="8">
+      <c r="A9" s="7">
         <v>8</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="6" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10" s="8">
+      <c r="A10" s="7">
         <v>9</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="6" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A11" s="8">
+      <c r="A11" s="7">
         <v>10</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="6" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A12" s="8">
+      <c r="A12" s="7">
         <v>11</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="6" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A13" s="8">
+      <c r="A13" s="7">
         <v>12</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A14" s="8">
+      <c r="A14" s="7">
         <v>13</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="6" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A15" s="8">
+      <c r="A15" s="7">
         <v>14</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="6" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A16" s="8">
+      <c r="A16" s="7">
         <v>15</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="6" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A17" s="8">
+      <c r="A17" s="7">
         <v>16</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="6" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A18" s="8">
+      <c r="A18" s="7">
         <v>17</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="6" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A19" s="8">
+      <c r="A19" s="7">
         <v>18</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="6" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A20" s="8">
+      <c r="A20" s="7">
         <v>19</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="6" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A21" s="8">
+      <c r="A21" s="7">
         <v>20</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="6" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A22" s="8">
+      <c r="A22" s="7">
         <v>21</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="6" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A23" s="8">
+      <c r="A23" s="7">
         <v>22</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="6" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A24" s="8">
+      <c r="A24" s="7">
         <v>23</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="6" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A25" s="8">
+      <c r="A25" s="7">
         <v>24</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="6" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A26" s="8">
+      <c r="A26" s="7">
         <v>25</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="6" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A27" s="8">
+      <c r="A27" s="7">
         <v>26</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D27" s="6" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A28" s="8">
+      <c r="A28" s="7">
         <v>27</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A29" s="8">
+      <c r="A29" s="7">
         <v>28</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="B29" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D29" s="6" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A30" s="8">
+      <c r="A30" s="7">
         <v>29</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="6" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A31" s="8">
+      <c r="A31" s="7">
         <v>30</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="B31" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="D31" s="6" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A32" s="8">
+      <c r="A32" s="7">
         <v>31</v>
       </c>
-      <c r="B32" s="9" t="s">
+      <c r="B32" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C32" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="D32" s="6" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A33" s="8">
+      <c r="A33" s="7">
         <v>32</v>
       </c>
-      <c r="B33" s="9" t="s">
+      <c r="B33" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="D33" s="7" t="s">
+      <c r="D33" s="6" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A34" s="8">
+      <c r="A34" s="7">
         <v>33</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="B34" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="D34" s="6" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A35" s="8">
+      <c r="A35" s="7">
         <v>34</v>
       </c>
-      <c r="B35" s="9" t="s">
+      <c r="B35" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="D35" s="6" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A36" s="8">
+      <c r="A36" s="7">
         <v>35</v>
       </c>
-      <c r="B36" s="9" t="s">
+      <c r="B36" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="C36" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="D36" s="7" t="s">
+      <c r="D36" s="6" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A37" s="8">
+      <c r="A37" s="7">
         <v>36</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="B37" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="C37" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="D37" s="7" t="s">
+      <c r="D37" s="6" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A38" s="8">
+      <c r="A38" s="7">
         <v>37</v>
       </c>
-      <c r="B38" s="9" t="s">
+      <c r="B38" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C38" s="4" t="s">
+      <c r="C38" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="D38" s="6" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A39" s="8">
+      <c r="A39" s="7">
         <v>38</v>
       </c>
-      <c r="B39" s="9" t="s">
+      <c r="B39" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C39" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="D39" s="7" t="s">
+      <c r="D39" s="6" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A40" s="8">
+      <c r="A40" s="7">
         <v>39</v>
       </c>
-      <c r="B40" s="9" t="s">
+      <c r="B40" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="C40" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="D40" s="7" t="s">
+      <c r="D40" s="6" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A41" s="8">
+      <c r="A41" s="7">
         <v>40</v>
       </c>
-      <c r="B41" s="9" t="s">
+      <c r="B41" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="C41" s="4" t="s">
+      <c r="C41" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="D41" s="7" t="s">
+      <c r="D41" s="6" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A42" s="8">
+      <c r="A42" s="7">
         <v>41</v>
       </c>
-      <c r="B42" s="9" t="s">
+      <c r="B42" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C42" s="4" t="s">
+      <c r="C42" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="D42" s="7" t="s">
+      <c r="D42" s="6" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A43" s="8">
+      <c r="A43" s="7">
         <v>42</v>
       </c>
-      <c r="B43" s="9" t="s">
+      <c r="B43" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="C43" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="D43" s="7" t="s">
+      <c r="D43" s="6" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A44" s="8">
+      <c r="A44" s="7">
         <v>43</v>
       </c>
-      <c r="B44" s="9" t="s">
+      <c r="B44" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C44" s="4" t="s">
+      <c r="C44" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="D44" s="7" t="s">
+      <c r="D44" s="6" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A45" s="8">
+      <c r="A45" s="7">
         <v>44</v>
       </c>
-      <c r="B45" s="9" t="s">
+      <c r="B45" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C45" s="4" t="s">
+      <c r="C45" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D45" s="7" t="s">
+      <c r="D45" s="6" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A46" s="8">
+      <c r="A46" s="7">
         <v>45</v>
       </c>
-      <c r="B46" s="9" t="s">
+      <c r="B46" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="C46" s="4" t="s">
+      <c r="C46" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="D46" s="7" t="s">
+      <c r="D46" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A47" s="8">
+      <c r="A47" s="7">
         <v>46</v>
       </c>
-      <c r="B47" s="9" t="s">
+      <c r="B47" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C47" s="4" t="s">
+      <c r="C47" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="D47" s="7" t="s">
+      <c r="D47" s="6" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B48" s="9"/>
+      <c r="B48" s="8"/>
     </row>
     <row r="49" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B49" s="9"/>
+      <c r="B49" s="8"/>
     </row>
     <row r="50" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B50" s="9"/>
+      <c r="B50" s="8"/>
     </row>
     <row r="51" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B51" s="9"/>
+      <c r="B51" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1711,91 +1714,91 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A1" s="14"/>
-      <c r="B1" s="11" t="s">
+      <c r="A1" s="13"/>
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="L1" s="11" t="s">
+      <c r="L1" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="M1" s="11" t="s">
+      <c r="M1" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="N1" s="11" t="s">
+      <c r="N1" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="O1" s="11" t="s">
+      <c r="O1" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="P1" s="11" t="s">
+      <c r="P1" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="Q1" s="11" t="s">
+      <c r="Q1" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="R1" s="11" t="s">
+      <c r="R1" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="S1" s="11" t="s">
+      <c r="S1" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="T1" s="11" t="s">
+      <c r="T1" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="U1" s="11" t="s">
+      <c r="U1" s="10" t="s">
         <v>172</v>
       </c>
-      <c r="V1" s="11" t="s">
+      <c r="V1" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="W1" s="11" t="s">
+      <c r="W1" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="X1" s="11" t="s">
+      <c r="X1" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="Y1" s="11" t="s">
+      <c r="Y1" s="10" t="s">
         <v>175</v>
       </c>
-      <c r="Z1" s="11" t="s">
+      <c r="Z1" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="AA1" s="11" t="s">
+      <c r="AA1" s="10" t="s">
         <v>176</v>
       </c>
-      <c r="AB1" s="11" t="s">
+      <c r="AB1" s="10" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="11" t="s">
         <v>115</v>
       </c>
       <c r="B2" s="1">
@@ -1831,7 +1834,7 @@
       <c r="AB2" s="1"/>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="11" t="s">
         <v>116</v>
       </c>
       <c r="B3" s="1"/>
@@ -1867,7 +1870,7 @@
       <c r="AB3" s="1"/>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="11" t="s">
         <v>117</v>
       </c>
       <c r="B4" s="1"/>
@@ -1909,7 +1912,7 @@
       <c r="AB4" s="1"/>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="11" t="s">
         <v>118</v>
       </c>
       <c r="B5" s="1"/>
@@ -1963,7 +1966,7 @@
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="11" t="s">
         <v>119</v>
       </c>
       <c r="B6" s="1"/>
@@ -1999,7 +2002,7 @@
       <c r="AB6" s="1"/>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="11" t="s">
         <v>138</v>
       </c>
       <c r="B7" s="1"/>
@@ -2033,7 +2036,7 @@
       <c r="AB7" s="1"/>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="11" t="s">
         <v>121</v>
       </c>
       <c r="B8" s="1"/>
@@ -2067,7 +2070,7 @@
       <c r="AB8" s="1"/>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="11" t="s">
         <v>122</v>
       </c>
       <c r="B9" s="1"/>
@@ -2101,7 +2104,7 @@
       <c r="AB9" s="1"/>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="11" t="s">
         <v>123</v>
       </c>
       <c r="B10" s="1"/>
@@ -2139,7 +2142,7 @@
       <c r="AB10" s="1"/>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="11" t="s">
         <v>124</v>
       </c>
       <c r="B11" s="1"/>
@@ -2175,7 +2178,7 @@
       <c r="AB11" s="1"/>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="11" t="s">
         <v>125</v>
       </c>
       <c r="B12" s="1"/>
@@ -2211,7 +2214,7 @@
       <c r="AB12" s="1"/>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="11" t="s">
         <v>120</v>
       </c>
       <c r="B13" s="1"/>
@@ -2257,7 +2260,7 @@
       <c r="AB13" s="1"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="11" t="s">
         <v>126</v>
       </c>
       <c r="B14" s="1"/>
@@ -2303,7 +2306,7 @@
       <c r="AB14" s="1"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="11" t="s">
         <v>127</v>
       </c>
       <c r="B15" s="1"/>
@@ -2325,7 +2328,9 @@
         <v>25</v>
       </c>
       <c r="R15" s="1"/>
-      <c r="S15" s="1"/>
+      <c r="S15" s="1" t="s">
+        <v>171</v>
+      </c>
       <c r="T15" s="1"/>
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
@@ -2343,7 +2348,7 @@
       <c r="AB15" s="1"/>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="11" t="s">
         <v>128</v>
       </c>
       <c r="B16" s="1"/>
@@ -2385,7 +2390,7 @@
       </c>
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="11" t="s">
         <v>164</v>
       </c>
       <c r="B17" s="1"/>
@@ -2419,7 +2424,7 @@
       <c r="AB17" s="1"/>
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="11" t="s">
         <v>129</v>
       </c>
       <c r="B18" s="1"/>
@@ -2463,7 +2468,7 @@
       </c>
     </row>
     <row r="19" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="11" t="s">
         <v>127</v>
       </c>
       <c r="B19" s="1"/>
@@ -2483,9 +2488,7 @@
       <c r="P19" s="1"/>
       <c r="Q19" s="1"/>
       <c r="R19" s="1"/>
-      <c r="S19" s="1" t="s">
-        <v>171</v>
-      </c>
+      <c r="S19" s="1"/>
       <c r="T19" s="1"/>
       <c r="U19" s="1"/>
       <c r="V19" s="1"/>
@@ -2497,7 +2500,7 @@
       <c r="AB19" s="1"/>
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="11" t="s">
         <v>133</v>
       </c>
       <c r="B20" s="1"/>
@@ -2539,8 +2542,8 @@
       </c>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A21" s="12" t="s">
-        <v>119</v>
+      <c r="A21" s="11" t="s">
+        <v>177</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -2571,7 +2574,7 @@
       <c r="AB21" s="1"/>
     </row>
     <row r="22" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A22" s="12" t="s">
+      <c r="A22" s="11" t="s">
         <v>130</v>
       </c>
       <c r="B22" s="1"/>
@@ -2613,7 +2616,7 @@
       <c r="AB22" s="1"/>
     </row>
     <row r="23" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="11" t="s">
         <v>131</v>
       </c>
       <c r="B23" s="1"/>
@@ -2651,7 +2654,7 @@
       <c r="AB23" s="1"/>
     </row>
     <row r="24" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A24" s="12" t="s">
+      <c r="A24" s="11" t="s">
         <v>132</v>
       </c>
       <c r="B24" s="1"/>
@@ -2689,7 +2692,7 @@
       <c r="AB24" s="1"/>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="11" t="s">
         <v>134</v>
       </c>
       <c r="B25" s="1"/>
@@ -2727,7 +2730,7 @@
       <c r="AB25" s="1"/>
     </row>
     <row r="26" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A26" s="12" t="s">
+      <c r="A26" s="11" t="s">
         <v>174</v>
       </c>
       <c r="B26" s="1"/>
@@ -2765,7 +2768,7 @@
       <c r="AB26" s="1"/>
     </row>
     <row r="27" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="11" t="s">
         <v>135</v>
       </c>
       <c r="B27" s="1"/>
@@ -2799,7 +2802,7 @@
       <c r="AB27" s="1"/>
     </row>
     <row r="28" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A28" s="13"/>
+      <c r="A28" s="12"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>

</xml_diff>